<commit_message>
Updated upload and excel feature
</commit_message>
<xml_diff>
--- a/reports/candidate_report.xlsx
+++ b/reports/candidate_report.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -548,36 +548,36 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Atiq ur Rehman</t>
+          <t>ALI RAZA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>atiq_78664@yahoo.com</t>
+          <t>ra635036@gmail.com</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Bachelor</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Customer Service, Operations, Restaurant Management</t>
+          <t>Leadership, Customer Service, Team Management, Operations, Restaurant Management, Communication, Cash Handling</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>23.07</v>
+        <v>21.43</v>
       </c>
       <c r="J5" t="n">
-        <v>36.64</v>
+        <v>42.06</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Selected</t>
         </is>
       </c>
     </row>
@@ -587,36 +587,36 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Zakaria Liaqat Ali</t>
+          <t>Atiq ur Rehman</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Zghory1@gmail.com</t>
+          <t>atiq_78664@yahoo.com</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Leadership, Customer Service, Communication, Cash Handling</t>
+          <t>Customer Service, Operations, Restaurant Management</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>16.21</v>
+        <v>20.72</v>
       </c>
       <c r="J6" t="n">
-        <v>30.12</v>
+        <v>35.23</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Selected</t>
         </is>
       </c>
     </row>
@@ -626,22 +626,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kashif Mehmood</t>
+          <t>AKHTAR ALI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cmkashif82@gmail.com</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>+923105605270</t>
+          <t>consultantdxb1@gmail.com</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -649,18 +644,18 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Customer Service, Food Safety, Communication</t>
+          <t>Leadership, Customer Service, Team Management, Inventory Management, Food Safety, Operations, Communication, Cash Handling</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>13.4</v>
+        <v>25.07</v>
       </c>
       <c r="J7" t="n">
-        <v>20.84</v>
+        <v>33.84</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Interview</t>
         </is>
       </c>
     </row>
@@ -670,36 +665,36 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MUNAHIL MAHMOOD</t>
+          <t>MUHAMMAD HASEEB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>munahilmehmood2@gmail.com</t>
+          <t>haseebabbasi964@gmail.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>BS</t>
+          <t>Bachelor</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Leadership, Food Safety, Operations, Communication</t>
+          <t>Leadership, Customer Service, Inventory Management, Food Safety, Operations</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>10.38</v>
+        <v>16</v>
       </c>
       <c r="J8" t="n">
-        <v>18.63</v>
+        <v>29.6</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Selected</t>
         </is>
       </c>
     </row>
@@ -709,39 +704,36 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RAHIB</t>
+          <t>Zakaria Liaqat Ali</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>siddiquirahib173@gmail.com</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>20</v>
+          <t>Zghory1@gmail.com</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>BS</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Leadership</t>
+          <t>Leadership, Customer Service, Communication, Cash Handling</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>5.54</v>
+        <v>14.62</v>
       </c>
       <c r="J9" t="n">
-        <v>14.93</v>
+        <v>29.17</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Selected</t>
         </is>
       </c>
     </row>
@@ -751,24 +743,190 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Kashif Mehmood</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>cmkashif82@gmail.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+923105605270</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Customer Service, Food Safety, Communication</t>
+        </is>
+      </c>
       <c r="I10" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="J10" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MUNAHIL MAHMOOD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>munahilmehmood2@gmail.com</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="n">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Leadership, Food Safety, Operations, Communication</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J11" t="n">
+        <v>18.88</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>KIRAN</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kiranainee54@gmail.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>03238225567</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J12" t="n">
+        <v>18.53</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Program 2026-27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>eh888313@gamil.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>03188421294</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
         <v>0</v>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>

</xml_diff>